<commit_message>
feat(trivy): repo + IaC config + secret scan 추가 — 자동 항목 4개 확장
- trivy-wrapper: /scan/repo, /scan/config, /scan/secret 신규 엔드포인트
  GitHub repo URL을 trivy CLI(repo / config / secret 서브커맨드)로 직접 처리
- validators: validate_trivy_repo + validate_trivy_target 추가
  이미지 참조 / GitHub URL / owner/repo 단축형 자동 판별
- trivy_collector: 4개 신규 함수 (autodiscover docstring 매핑)
  5.4.1.1_1 collect_repo_vuln_scan        — repo Critical+High 취약점
  5.5.1.1_1 collect_source_secret_scan    — 노출된 secret 검출
  5.5.1.1_2 collect_iac_misconfig_scan    — Dockerfile/k8s/Terraform 위반
  5.5.2.1_1 collect_repo_risk_identification — 위험 요소 자동 식별
- zt-checklist.xlsx: 위 4개 항목을 수동→자동(Trivy)로 마이그레이션 + 판정/추출/로직 갱신
- frontend NewAssessment: 입력란 라벨 "컨테이너 이미지 또는 GitHub repo (Trivy)"
  placeholder + helper text 갱신

매핑 검증: xlsx 자동 216 ↔ 우리 매핑 unique 216 (1:1 정합). 잘못/누락/충돌 0건.
도구별: keycloak 65 / wazuh 122 / nmap 14 / trivy 15 = 216

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/zt-checklist.xlsx
+++ b/backend/zt-checklist.xlsx
@@ -13316,42 +13316,42 @@
       </c>
       <c r="D219" s="15" t="inlineStr">
         <is>
-          <t>애플리케이션 배포 전 수동으로 코드 검토 및 취약점 검사를 수행하는가?</t>
+          <t>GitHub repo 소스 코드에 대한 자동 취약점 스캔이 수행되는가?</t>
         </is>
       </c>
       <c r="E219" s="21" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="F219" s="22" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>Trivy (래퍼 필요)</t>
         </is>
       </c>
       <c r="G219" s="15" t="inlineStr">
         <is>
-          <t>수동 코드 검토·취약점 점검 기록 존재 여부</t>
+          <t>trivy repo 스캔 결과 (Critical/High 취약점 수)</t>
         </is>
       </c>
       <c r="H219" s="15" t="inlineStr">
         <is>
-          <t>기록 존재 → 충족 / 미존재 → 미충족</t>
+          <t>스캔 수행 AND Critical+High = 0 → 충족 / Critical+High ≤ 5 → 부분 충족 / 그 외 → 미충족</t>
         </is>
       </c>
       <c r="I219" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>severity_counts.CRITICAL, severity_counts.HIGH (per package)</t>
         </is>
       </c>
       <c r="J219" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>분자: CRITICAL+HIGH 합계, 분모: 1 (지표=절대수)</t>
         </is>
       </c>
       <c r="K219" s="20" t="inlineStr">
         <is>
-          <t>증빙 미제출 → 미충족</t>
+          <t>저장소 미입력/접근 불가 → 평가 불가 / 타임아웃(300초) → 평가 불가</t>
         </is>
       </c>
     </row>
@@ -14406,42 +14406,42 @@
       </c>
       <c r="D238" s="15" t="inlineStr">
         <is>
-          <t>개발 프로세스에 보안 코딩 표준이 적용되어 있는가?</t>
+          <t>소스 코드 내 노출된 비밀번호·API key·토큰이 자동 검출되어 차단되는가?</t>
         </is>
       </c>
       <c r="E238" s="21" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="F238" s="22" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>Trivy (래퍼 필요)</t>
         </is>
       </c>
       <c r="G238" s="15" t="inlineStr">
         <is>
-          <t>보안 코딩 표준 문서 존재 여부</t>
+          <t>trivy --scanners secret 스캔 결과 (노출 secret 수)</t>
         </is>
       </c>
       <c r="H238" s="15" t="inlineStr">
         <is>
-          <t>존재 → 충족 / 미존재 → 미충족</t>
+          <t>노출 secret = 0건 → 충족 / 1~3건 → 부분 충족 / 4건 이상 → 미충족</t>
         </is>
       </c>
       <c r="I238" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>secrets[].RuleID, secrets[].Severity, secrets[].Target</t>
         </is>
       </c>
       <c r="J238" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>분자: 검출된 secret 수, 분모: 1</t>
         </is>
       </c>
       <c r="K238" s="20" t="inlineStr">
         <is>
-          <t>증빙 미제출 → 미충족</t>
+          <t>저장소 미입력 → 평가 불가 / 타임아웃(300초) → 평가 불가</t>
         </is>
       </c>
     </row>
@@ -14463,42 +14463,42 @@
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
-          <t>코드 배포 전, 정적이고 수동으로 보안 테스트를 수행하는가?</t>
+          <t>IaC(Dockerfile/Kubernetes/Terraform) 설정 파일에 대한 정적 보안 분석이 자동화되어 있는가?</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="F239" s="8" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>Trivy (래퍼 필요)</t>
         </is>
       </c>
       <c r="G239" s="5" t="inlineStr">
         <is>
-          <t>정적 보안 테스트 기록 존재 여부</t>
+          <t>trivy config / repo --scanners misconfig 결과 (High+Critical 위반 수)</t>
         </is>
       </c>
       <c r="H239" s="5" t="inlineStr">
         <is>
-          <t>기록 존재 → 충족 / 미존재 → 미충족</t>
+          <t>High+Critical 위반 = 0 → 충족 / 1~5건 → 부분 충족 / 6건 이상 → 미충족</t>
         </is>
       </c>
       <c r="I239" s="9" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>Misconfigurations[].Severity, Misconfigurations[].ID</t>
         </is>
       </c>
       <c r="J239" s="9" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>분자: severity가 CRITICAL+HIGH인 misconfig 수, 분모: 1</t>
         </is>
       </c>
       <c r="K239" s="10" t="inlineStr">
         <is>
-          <t>증빙 미제출 → 미충족</t>
+          <t>저장소 미입력 → 평가 불가 / 타임아웃(300초) → 평가 불가</t>
         </is>
       </c>
     </row>
@@ -14978,42 +14978,42 @@
       </c>
       <c r="D248" s="15" t="inlineStr">
         <is>
-          <t>최소한의 위험 요소가 식별되고 문서화 하였는가?</t>
+          <t>소프트웨어 위험 요소(취약점·의존성·secret)가 자동 식별되어 가시화되는가?</t>
         </is>
       </c>
       <c r="E248" s="21" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>자동</t>
         </is>
       </c>
       <c r="F248" s="22" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>Trivy (래퍼 필요)</t>
         </is>
       </c>
       <c r="G248" s="15" t="inlineStr">
         <is>
-          <t>위험 요소 식별·문서화 자료 존재 여부</t>
+          <t>trivy repo 스캔의 component_count (식별된 위험 요소 수)</t>
         </is>
       </c>
       <c r="H248" s="15" t="inlineStr">
         <is>
-          <t>존재 → 충족 / 미존재 → 미충족</t>
+          <t>식별 결과 ≥ 1건(스캔 자체 수행) → 충족 / 스캔 실패 → 미충족</t>
         </is>
       </c>
       <c r="I248" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>Results[], severity_counts (집계)</t>
         </is>
       </c>
       <c r="J248" s="19" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>분자: 스캔 수행 여부(1/0), 분모: 1</t>
         </is>
       </c>
       <c r="K248" s="20" t="inlineStr">
         <is>
-          <t>증빙 미제출 → 미충족</t>
+          <t>저장소 미입력 → 평가 불가 / 타임아웃(300초) → 평가 불가</t>
         </is>
       </c>
     </row>
@@ -18708,7 +18708,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="34" t="inlineStr">
         <is>
@@ -18793,7 +18792,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="34" t="inlineStr">
         <is>

</xml_diff>